<commit_message>
feat(security,ui): whitelist SQL console access, sober enterprise dashboard redesign
- server.py: replace SQL keyword-blocklist with table whitelist + CTE support,
  add real query timeout via thread interrupt (DuckDB has no statement_timeout),
  cap unbounded results with an implicit LIMIT.
- templates/index.html: full visual redesign (top nav instead of dark sidebar,
  neutral stone palette with a single muted copper accent, Manrope + IBM Plex Mono),
  escape SQL console output to close a reflected-XSS gap.
- Reorganize deep audit/process docs into anexos_avanzados/ (reference material,
  not part of the main case study) and drop the internal PROJECT_TRACKER.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entregables_planta/Matriz_SMED_Reduccion_Setups.xlsx
+++ b/entregables_planta/Matriz_SMED_Reduccion_Setups.xlsx
@@ -10,7 +10,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_SMED_Llenadora" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen_Etapas_Shingo" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impacto_Financiero_Planta" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria_AMFE_Riesgos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +24,7 @@
     <numFmt numFmtId="166" formatCode="0.0 &quot;min&quot;"/>
     <numFmt numFmtId="167" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,41 +59,8 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <i val="1"/>
-      <color rgb="00333333"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -119,38 +85,8 @@
         <bgColor rgb="00B4C6E7"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B365D"/>
-        <bgColor rgb="001B365D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00008080"/>
-        <bgColor rgb="00008080"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002C3E50"/>
-        <bgColor rgb="002C3E50"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FADBD8"/>
-        <bgColor rgb="00FADBD8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4EFDF"/>
-        <bgColor rgb="00D4EFDF"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -186,25 +122,11 @@
         <color rgb="001F4E78"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9D9D9"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -257,48 +179,6 @@
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1867,7 +1747,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>Inversión Requerida (Utillajes Tri-Clamp, Carros 5S, Galgas)</t>
+          <t>Inversión Requerida (Cabezal sanitario, tanque encamisado, kit de cambio rápido)</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1879,14 +1759,14 @@
         <v>0</v>
       </c>
       <c r="D17" s="20" t="n">
-        <v>4800</v>
+        <v>23800</v>
       </c>
       <c r="E17" s="20" t="n">
-        <v>4800</v>
+        <v>23800</v>
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Capex Cero (Gasto menor OPEX de utillaje rápido)</t>
+          <t>Capex menor (frente a $250k de una línea nueva)</t>
         </is>
       </c>
     </row>
@@ -1905,14 +1785,14 @@
         <v>0</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>3</v>
+        <v>14.9</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>-3</v>
+        <v>-14.9</v>
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>($4,800 / $581,609 anual) * 365 días = 3 días</t>
+          <t>($23,800 / $581,609 anual) * 365 días = 14.9 días</t>
         </is>
       </c>
     </row>
@@ -1945,743 +1825,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>AUDITORÍA INTEGRAL PRE-MORTEM: MATRIZ AMFE (FMEA) Y ANÁLISIS DE RIESGOS EN PLANTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>Evaluación Forense de Modos de Falla: Desacople Térmico de Horno, Bloqueo de Encartonadora, Seguridad Alimentaria (ATP) y Presupuesto Real</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="23" t="inlineStr">
-        <is>
-          <t>1. MATRIZ AMFE (FMEA) DE PROCESO: ANÁLISIS CUANTITATIVO DE MODOS DE FALLA EN SMED</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B5" s="24" t="inlineStr">
-        <is>
-          <t>Modo de Falla Potencial</t>
-        </is>
-      </c>
-      <c r="C5" s="24" t="inlineStr">
-        <is>
-          <t>Causa Raíz Operacional</t>
-        </is>
-      </c>
-      <c r="D5" s="24" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E5" s="24" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="F5" s="24" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="G5" s="24" t="inlineStr">
-        <is>
-          <t>NPR Inicial</t>
-        </is>
-      </c>
-      <c r="H5" s="24" t="inlineStr">
-        <is>
-          <t>Contramedida de Ingeniería Blindada</t>
-        </is>
-      </c>
-      <c r="I5" s="24" t="inlineStr">
-        <is>
-          <t>S*</t>
-        </is>
-      </c>
-      <c r="J5" s="24" t="inlineStr">
-        <is>
-          <t>O*</t>
-        </is>
-      </c>
-      <c r="K5" s="24" t="inlineStr">
-        <is>
-          <t>NPR Final</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="25" t="inlineStr">
-        <is>
-          <t>MF-01</t>
-        </is>
-      </c>
-      <c r="B6" s="26" t="inlineStr">
-        <is>
-          <t>Inercia Térmica del Horno Túnel (Starvation)</t>
-        </is>
-      </c>
-      <c r="C6" s="26" t="inlineStr">
-        <is>
-          <t>Horno tarda 35 min en estabilizar T; llenadora lista a los 15 min queda vacía</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="E6" s="25" t="n">
-        <v>8</v>
-      </c>
-      <c r="F6" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="27">
-        <f>D6*E6*F6</f>
-        <v/>
-      </c>
-      <c r="H6" s="26" t="inlineStr">
-        <is>
-          <t>Programación Heijunka con menor delta T y preaviso a quemadores 20 min antes</t>
-        </is>
-      </c>
-      <c r="I6" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="J6" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" s="28">
-        <f>I6*J6*2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="25" t="inlineStr">
-        <is>
-          <t>MF-02</t>
-        </is>
-      </c>
-      <c r="B7" s="26" t="inlineStr">
-        <is>
-          <t>Bloqueo por Encartonadora (Downstream Choke)</t>
-        </is>
-      </c>
-      <c r="C7" s="26" t="inlineStr">
-        <is>
-          <t>Encartonadora tarda hasta 276 min en formato; buffer de 3 min colapsa la llenadora</t>
-        </is>
-      </c>
-      <c r="D7" s="25" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="F7" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="27">
-        <f>D7*E7*F7</f>
-        <v/>
-      </c>
-      <c r="H7" s="26" t="inlineStr">
-        <is>
-          <t>SMED simultáneo en encartonadora con galgas de ajuste rápido y control de flujo</t>
-        </is>
-      </c>
-      <c r="I7" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="J7" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="K7" s="28">
-        <f>I7*J7*2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="25" t="inlineStr">
-        <is>
-          <t>MF-03</t>
-        </is>
-      </c>
-      <c r="B8" s="26" t="inlineStr">
-        <is>
-          <t>Contaminación Cruzada por Alérgenos</t>
-        </is>
-      </c>
-      <c r="C8" s="26" t="inlineStr">
-        <is>
-          <t>Arranque a los 15 min sin validación de QA; trazas de leche en galleta sin alérgeno</t>
-        </is>
-      </c>
-      <c r="D8" s="25" t="n">
-        <v>10</v>
-      </c>
-      <c r="E8" s="25" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="G8" s="27">
-        <f>D8*E8*F8</f>
-        <v/>
-      </c>
-      <c r="H8" s="26" t="inlineStr">
-        <is>
-          <t>Protocolo ATP al minuto 12 con luminómetro digital (&lt;30 RLU); firma digital obligatoria</t>
-        </is>
-      </c>
-      <c r="I8" s="25" t="n">
-        <v>9</v>
-      </c>
-      <c r="J8" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="28">
-        <f>I8*J8*2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="25" t="inlineStr">
-        <is>
-          <t>MF-04</t>
-        </is>
-      </c>
-      <c r="B9" s="26" t="inlineStr">
-        <is>
-          <t>Proliferación Bacteriana en Cabezal Gemelo</t>
-        </is>
-      </c>
-      <c r="C9" s="26" t="inlineStr">
-        <is>
-          <t>Cabezal lavado almacenado húmedo a 22°C incuba biofilm y Listeria monocytogenes</t>
-        </is>
-      </c>
-      <c r="D9" s="25" t="n">
-        <v>9</v>
-      </c>
-      <c r="E9" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="G9" s="27">
-        <f>D9*E9*F9</f>
-        <v/>
-      </c>
-      <c r="H9" s="26" t="inlineStr">
-        <is>
-          <t>Secado con aire HEPA 0.01um, desinfección alcohólica 70% y bolsa sellada con vencimiento 24h</t>
-        </is>
-      </c>
-      <c r="I9" s="25" t="n">
-        <v>8</v>
-      </c>
-      <c r="J9" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="28">
-        <f>I9*J9*2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>MF-05</t>
-        </is>
-      </c>
-      <c r="B10" s="26" t="inlineStr">
-        <is>
-          <t>Sinéresis y Choque Térmico de Crema</t>
-        </is>
-      </c>
-      <c r="C10" s="26" t="inlineStr">
-        <is>
-          <t>Crema a 28°C sin agitación se separa; boquillas frías provocan cristalización alfa</t>
-        </is>
-      </c>
-      <c r="D10" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="25" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="27">
-        <f>D10*E10*F10</f>
-        <v/>
-      </c>
-      <c r="H10" s="26" t="inlineStr">
-        <is>
-          <t>Tanque encamisado a 30°C con raspador continuo a 15 RPM y manta térmica en carro 5S</t>
-        </is>
-      </c>
-      <c r="I10" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="K10" s="28">
-        <f>I10*J10*2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="25" t="inlineStr">
-        <is>
-          <t>MF-06</t>
-        </is>
-      </c>
-      <c r="B11" s="26" t="inlineStr">
-        <is>
-          <t>Lesión Lumbar por Carga de Cabezal</t>
-        </is>
-      </c>
-      <c r="C11" s="26" t="inlineStr">
-        <is>
-          <t>Operador levanta solo un bloque de 32 kg excediendo límite NIOSH (Lifting Index 2.85)</t>
-        </is>
-      </c>
-      <c r="D11" s="25" t="n">
-        <v>8</v>
-      </c>
-      <c r="E11" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="F11" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="G11" s="27">
-        <f>D11*E11*F11</f>
-        <v/>
-      </c>
-      <c r="H11" s="26" t="inlineStr">
-        <is>
-          <t>Montaje obligatorio a cuatro manos y brazo pescante articulado de gravedad cero</t>
-        </is>
-      </c>
-      <c r="I11" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" s="28">
-        <f>I11*J11*1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="25" t="inlineStr">
-        <is>
-          <t>MF-07</t>
-        </is>
-      </c>
-      <c r="B12" s="26" t="inlineStr">
-        <is>
-          <t>Saturación de Almacén de Producto Terminado</t>
-        </is>
-      </c>
-      <c r="C12" s="26" t="inlineStr">
-        <is>
-          <t>271 pallets/mes adicionales saturan bodega si demanda comercial no los absorbe</t>
-        </is>
-      </c>
-      <c r="D12" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" s="25" t="n">
-        <v>7</v>
-      </c>
-      <c r="F12" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="G12" s="27">
-        <f>D12*E12*F12</f>
-        <v/>
-      </c>
-      <c r="H12" s="26" t="inlineStr">
-        <is>
-          <t>Alineación quincenal S&amp;OP, lotes nivelados y contratos de distribución ágiles</t>
-        </is>
-      </c>
-      <c r="I12" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="J12" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="28">
-        <f>I12*J12*2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="23" t="inlineStr">
-        <is>
-          <t>2. PRESUPUESTO REAL DE INGENIERÍA Y ADQUISICIONES AUDITADO (CAPEX DEFENDIBLE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="29" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B15" s="29" t="inlineStr">
-        <is>
-          <t>Descripción del Activo / Dispositivo Sanitario</t>
-        </is>
-      </c>
-      <c r="D15" s="29" t="inlineStr">
-        <is>
-          <t>Especificación Técnica de Ingeniería</t>
-        </is>
-      </c>
-      <c r="F15" s="29" t="inlineStr">
-        <is>
-          <t>Costo Fase 3 (Inicial)</t>
-        </is>
-      </c>
-      <c r="G15" s="29" t="inlineStr">
-        <is>
-          <t>Costo Auditado (Real)</t>
-        </is>
-      </c>
-      <c r="H15" s="29" t="inlineStr">
-        <is>
-          <t>Delta ($ USD)</t>
-        </is>
-      </c>
-      <c r="I15" s="29" t="inlineStr">
-        <is>
-          <t>Justificación Técnica de Auditoría</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B16" s="26" t="inlineStr">
-        <is>
-          <t>Cabezal Gemelo de Boquillas</t>
-        </is>
-      </c>
-      <c r="C16" s="30" t="n"/>
-      <c r="D16" s="26" t="inlineStr">
-        <is>
-          <t>Monobloque CNC en acero inoxidable AISI 316L con 12 pistones de precisión</t>
-        </is>
-      </c>
-      <c r="E16" s="30" t="n"/>
-      <c r="F16" s="31" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G16" s="31" t="n">
-        <v>9500</v>
-      </c>
-      <c r="H16" s="31">
-        <f>G16-F16</f>
-        <v/>
-      </c>
-      <c r="I16" s="26" t="inlineStr">
-        <is>
-          <t>Costos reales de mecanizado sanitario de alta precisión para alimentos</t>
-        </is>
-      </c>
-      <c r="J16" s="30" t="n"/>
-      <c r="K16" s="30" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B17" s="26" t="inlineStr">
-        <is>
-          <t>Tanque Pulmón Encamisado</t>
-        </is>
-      </c>
-      <c r="C17" s="30" t="n"/>
-      <c r="D17" s="26" t="inlineStr">
-        <is>
-          <t>Tanque móvil de 150L con camisa eléctrica a 30°C y raspador de bajas RPM</t>
-        </is>
-      </c>
-      <c r="E17" s="30" t="n"/>
-      <c r="F17" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="31" t="n">
-        <v>5200</v>
-      </c>
-      <c r="H17" s="31">
-        <f>G17-F17</f>
-        <v/>
-      </c>
-      <c r="I17" s="26" t="inlineStr">
-        <is>
-          <t>Evita la sinéresis y la separación de grasas en la crema de relleno</t>
-        </is>
-      </c>
-      <c r="J17" s="30" t="n"/>
-      <c r="K17" s="30" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="25" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B18" s="26" t="inlineStr">
-        <is>
-          <t>Brazo Pescante Ergonómico</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="n"/>
-      <c r="D18" s="26" t="inlineStr">
-        <is>
-          <t>Polipasto neumático balanceado de gravedad cero anclado a estructura</t>
-        </is>
-      </c>
-      <c r="E18" s="30" t="n"/>
-      <c r="F18" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="31" t="n">
-        <v>3800</v>
-      </c>
-      <c r="H18" s="31">
-        <f>G18-F18</f>
-        <v/>
-      </c>
-      <c r="I18" s="26" t="inlineStr">
-        <is>
-          <t>Cumplimiento estricto de norma NIOSH / ISO 11228-1 para carga de 32 kg</t>
-        </is>
-      </c>
-      <c r="J18" s="30" t="n"/>
-      <c r="K18" s="30" t="n"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="25" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B19" s="26" t="inlineStr">
-        <is>
-          <t>Carro Móvil 5S Sanitario</t>
-        </is>
-      </c>
-      <c r="C19" s="30" t="n"/>
-      <c r="D19" s="26" t="inlineStr">
-        <is>
-          <t>Estructura en acero inoxidable con manta calefactora para atemperar utillaje</t>
-        </is>
-      </c>
-      <c r="E19" s="30" t="n"/>
-      <c r="F19" s="31" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G19" s="31" t="n">
-        <v>2100</v>
-      </c>
-      <c r="H19" s="31">
-        <f>G19-F19</f>
-        <v/>
-      </c>
-      <c r="I19" s="26" t="inlineStr">
-        <is>
-          <t>Incluye sistema térmico para evitar choque frío en boquillas dosificadoras</t>
-        </is>
-      </c>
-      <c r="J19" s="30" t="n"/>
-      <c r="K19" s="30" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="25" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B20" s="26" t="inlineStr">
-        <is>
-          <t>Galgas Poka-Yoke y Tri-Clamps</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="n"/>
-      <c r="D20" s="26" t="inlineStr">
-        <is>
-          <t>6 galgas rectificadas de precisión + 8 abrazaderas Tri-Clamp sanitarias 3A</t>
-        </is>
-      </c>
-      <c r="E20" s="30" t="n"/>
-      <c r="F20" s="31" t="n">
-        <v>800</v>
-      </c>
-      <c r="G20" s="31" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H20" s="31">
-        <f>G20-F20</f>
-        <v/>
-      </c>
-      <c r="I20" s="26" t="inlineStr">
-        <is>
-          <t>Abrazaderas con certificación 3A para contacto directo con alimentos</t>
-        </is>
-      </c>
-      <c r="J20" s="30" t="n"/>
-      <c r="K20" s="30" t="n"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="25" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B21" s="26" t="inlineStr">
-        <is>
-          <t>Luminómetro Digital ATP y Swabs</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="n"/>
-      <c r="D21" s="26" t="inlineStr">
-        <is>
-          <t>Equipo Hygiena EnSURE Touch + 200 hisopos UltraSnap de bioluminiscencia</t>
-        </is>
-      </c>
-      <c r="E21" s="30" t="n"/>
-      <c r="F21" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="31" t="n">
-        <v>2000</v>
-      </c>
-      <c r="H21" s="31">
-        <f>G21-F21</f>
-        <v/>
-      </c>
-      <c r="I21" s="26" t="inlineStr">
-        <is>
-          <t>Garantiza liberación microbiológica formal en 2 minutos antes de arrancar</t>
-        </is>
-      </c>
-      <c r="J21" s="30" t="n"/>
-      <c r="K21" s="30" t="n"/>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="32" t="inlineStr">
-        <is>
-          <t>TOTAL INVERSIÓN DE PROYECTO AUDITADA</t>
-        </is>
-      </c>
-      <c r="B22" s="33" t="n"/>
-      <c r="C22" s="33" t="n"/>
-      <c r="D22" s="33" t="n"/>
-      <c r="E22" s="33" t="n"/>
-      <c r="F22" s="34">
-        <f>SUM(F16:F21)</f>
-        <v/>
-      </c>
-      <c r="G22" s="35">
-        <f>SUM(G16:G21)</f>
-        <v/>
-      </c>
-      <c r="H22" s="34">
-        <f>SUM(H16:H21)</f>
-        <v/>
-      </c>
-      <c r="I22" s="36" t="inlineStr">
-        <is>
-          <t>Payback Auditado: 14.9 Días (Frente a 9 meses de una línea nueva de )</t>
-        </is>
-      </c>
-      <c r="J22" s="33" t="n"/>
-      <c r="K22" s="33" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="A14:K14"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="I15:K15"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="B20:C20"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>